<commit_message>
Daily recap, matchup updates, learning and research 2026-08-22
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-22.xlsx
+++ b/data/k-props/2026-08-22.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="98">
   <si>
     <t>date</t>
   </si>
@@ -145,24 +145,33 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>&gt;=7</t>
+  </si>
+  <si>
+    <t>Ryan Weathers</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Martín Pérez</t>
+  </si>
+  <si>
+    <t>Atlanta Braves @ Milwaukee Brewers</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>Ryan Weathers</t>
-  </si>
-  <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Martín Pérez</t>
-  </si>
-  <si>
-    <t>Atlanta Braves @ Milwaukee Brewers</t>
-  </si>
-  <si>
     <t>Logan Henderson</t>
   </si>
   <si>
@@ -170,6 +179,9 @@
   </si>
   <si>
     <t>Washington Nationals @ Miami Marlins</t>
+  </si>
+  <si>
+    <t>O</t>
   </si>
   <si>
     <t>Eury Pérez</t>
@@ -874,17 +886,23 @@
       <c r="Y2">
         <v>1.0348</v>
       </c>
+      <c r="Z2">
+        <v>8</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>2.55</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>11.05</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.3546</v>
@@ -894,6 +912,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>-3.05</v>
+      </c>
+      <c r="AJ2">
+        <v>3.05</v>
+      </c>
+      <c r="AK2">
+        <v>-3.05</v>
+      </c>
+      <c r="AL2">
+        <v>3.05</v>
       </c>
       <c r="AM2">
         <v>11.05</v>
@@ -904,7 +934,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>5.5</v>
@@ -975,17 +1005,23 @@
       <c r="Y3">
         <v>0.943</v>
       </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>-1.15</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>4.35</v>
       </c>
       <c r="AE3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF3">
         <v>0.2287</v>
@@ -995,6 +1031,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-1.35</v>
+      </c>
+      <c r="AJ3">
+        <v>1.35</v>
+      </c>
+      <c r="AK3">
+        <v>-1.35</v>
+      </c>
+      <c r="AL3">
+        <v>1.35</v>
       </c>
       <c r="AM3">
         <v>4.35</v>
@@ -1005,10 +1053,10 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G4">
         <v>823743</v>
@@ -1068,16 +1116,16 @@
         <v>0.9813</v>
       </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD4">
         <v>3.6</v>
       </c>
       <c r="AE4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF4">
         <v>0.1715</v>
@@ -1097,7 +1145,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C5">
         <v>6.5</v>
@@ -1109,7 +1157,7 @@
         <v>-112</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>823743</v>
@@ -1168,17 +1216,23 @@
       <c r="Y5">
         <v>0.9745</v>
       </c>
+      <c r="Z5">
+        <v>4</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>-0.65</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD5">
         <v>5.85</v>
       </c>
       <c r="AE5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF5">
         <v>0.2907</v>
@@ -1188,6 +1242,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>-1.85</v>
+      </c>
+      <c r="AJ5">
+        <v>1.85</v>
+      </c>
+      <c r="AK5">
+        <v>-1.85</v>
+      </c>
+      <c r="AL5">
+        <v>1.85</v>
       </c>
       <c r="AM5">
         <v>5.85</v>
@@ -1198,7 +1264,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C6">
         <v>2.5</v>
@@ -1210,7 +1276,7 @@
         <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>823831</v>
@@ -1269,17 +1335,23 @@
       <c r="Y6">
         <v>0.9201</v>
       </c>
+      <c r="Z6">
+        <v>4</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB6">
+        <v>1.55</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD6">
         <v>4.05</v>
       </c>
       <c r="AE6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF6">
         <v>0.2021</v>
@@ -1289,6 +1361,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>-0.05</v>
+      </c>
+      <c r="AJ6">
+        <v>0.05</v>
+      </c>
+      <c r="AK6">
+        <v>-0.05</v>
+      </c>
+      <c r="AL6">
+        <v>0.05</v>
       </c>
       <c r="AM6">
         <v>4.05</v>
@@ -1299,10 +1383,10 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>823831</v>
@@ -1362,16 +1446,16 @@
         <v>1.0251</v>
       </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD7">
         <v>6.81</v>
       </c>
       <c r="AE7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AF7">
         <v>0.2665</v>
@@ -1391,7 +1475,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1403,7 +1487,7 @@
         <v>128</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G8">
         <v>823422</v>
@@ -1462,17 +1546,23 @@
       <c r="Y8">
         <v>0.8933</v>
       </c>
+      <c r="Z8">
+        <v>8</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB8">
+        <v>-0.05</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD8">
         <v>3.45</v>
       </c>
       <c r="AE8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF8">
         <v>0.2027</v>
@@ -1482,6 +1572,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>4.55</v>
+      </c>
+      <c r="AJ8">
+        <v>4.55</v>
+      </c>
+      <c r="AK8">
+        <v>4.55</v>
+      </c>
+      <c r="AL8">
+        <v>4.55</v>
       </c>
       <c r="AM8">
         <v>3.45</v>
@@ -1492,7 +1594,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C9">
         <v>4.5</v>
@@ -1504,7 +1606,7 @@
         <v>-118</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>824798</v>
@@ -1563,17 +1665,23 @@
       <c r="Y9">
         <v>1.0352</v>
       </c>
+      <c r="Z9">
+        <v>5</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB9">
+        <v>0.19</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD9">
         <v>4.69</v>
       </c>
       <c r="AE9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF9">
         <v>0.2072</v>
@@ -1583,6 +1691,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>0.31</v>
+      </c>
+      <c r="AJ9">
+        <v>0.31</v>
+      </c>
+      <c r="AK9">
+        <v>0.31</v>
+      </c>
+      <c r="AL9">
+        <v>0.31</v>
       </c>
       <c r="AM9">
         <v>4.69</v>
@@ -1593,7 +1713,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C10">
         <v>3.5</v>
@@ -1605,7 +1725,7 @@
         <v>110</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>824798</v>
@@ -1664,17 +1784,23 @@
       <c r="Y10">
         <v>0.88</v>
       </c>
+      <c r="Z10">
+        <v>3</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-0.58</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD10">
         <v>2.92</v>
       </c>
       <c r="AE10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF10">
         <v>0.1776</v>
@@ -1684,6 +1810,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>0.08</v>
+      </c>
+      <c r="AJ10">
+        <v>0.08</v>
+      </c>
+      <c r="AK10">
+        <v>0.08</v>
+      </c>
+      <c r="AL10">
+        <v>0.08</v>
       </c>
       <c r="AM10">
         <v>2.92</v>
@@ -1694,7 +1832,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C11">
         <v>3.5</v>
@@ -1706,13 +1844,13 @@
         <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G11">
         <v>822858</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I11">
         <v>4.4</v>
@@ -1765,17 +1903,23 @@
       <c r="Y11">
         <v>1.0657</v>
       </c>
+      <c r="Z11">
+        <v>3</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>0.66</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD11">
         <v>4.16</v>
       </c>
       <c r="AE11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF11">
         <v>0.1638</v>
@@ -1785,6 +1929,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>-1.16</v>
+      </c>
+      <c r="AJ11">
+        <v>1.16</v>
+      </c>
+      <c r="AK11">
+        <v>-1.16</v>
+      </c>
+      <c r="AL11">
+        <v>1.16</v>
       </c>
       <c r="AM11">
         <v>4.16</v>
@@ -1795,7 +1951,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1807,13 +1963,13 @@
         <v>121</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G12">
         <v>822858</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I12">
         <v>4.3</v>
@@ -1866,17 +2022,23 @@
       <c r="Y12">
         <v>1.0991</v>
       </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>-0.37</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD12">
         <v>4.13</v>
       </c>
       <c r="AE12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF12">
         <v>0.1507</v>
@@ -1886,6 +2048,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>-1.13</v>
+      </c>
+      <c r="AJ12">
+        <v>1.13</v>
+      </c>
+      <c r="AK12">
+        <v>-1.13</v>
+      </c>
+      <c r="AL12">
+        <v>1.13</v>
       </c>
       <c r="AM12">
         <v>4.13</v>
@@ -1896,7 +2070,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1908,13 +2082,13 @@
         <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G13">
         <v>824151</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I13">
         <v>4.5</v>
@@ -1967,17 +2141,23 @@
       <c r="Y13">
         <v>0.9272</v>
       </c>
+      <c r="Z13">
+        <v>9</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB13">
+        <v>-0.5</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD13">
         <v>4</v>
       </c>
       <c r="AE13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF13">
         <v>0.2386</v>
@@ -1987,6 +2167,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>5</v>
+      </c>
+      <c r="AJ13">
+        <v>5</v>
+      </c>
+      <c r="AK13">
+        <v>5</v>
+      </c>
+      <c r="AL13">
+        <v>5</v>
       </c>
       <c r="AM13">
         <v>4</v>
@@ -1997,7 +2189,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -2009,7 +2201,7 @@
         <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>824151</v>
@@ -2068,17 +2260,23 @@
       <c r="Y14">
         <v>1.0455</v>
       </c>
+      <c r="Z14">
+        <v>4</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>-0.84</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD14">
         <v>4.66</v>
       </c>
       <c r="AE14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF14">
         <v>0.2384</v>
@@ -2088,6 +2286,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-0.66</v>
+      </c>
+      <c r="AJ14">
+        <v>0.66</v>
+      </c>
+      <c r="AK14">
+        <v>-0.66</v>
+      </c>
+      <c r="AL14">
+        <v>0.66</v>
       </c>
       <c r="AM14">
         <v>4.66</v>
@@ -2098,7 +2308,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>5.5</v>
@@ -2110,7 +2320,7 @@
         <v>126</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G15">
         <v>824560</v>
@@ -2169,17 +2379,23 @@
       <c r="Y15">
         <v>1.0743</v>
       </c>
+      <c r="Z15">
+        <v>6</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB15">
+        <v>1.12</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD15">
         <v>6.45</v>
       </c>
       <c r="AE15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AF15">
         <v>0.2853</v>
@@ -2189,6 +2405,18 @@
       </c>
       <c r="AH15">
         <v>0.17</v>
+      </c>
+      <c r="AI15">
+        <v>-0.45</v>
+      </c>
+      <c r="AJ15">
+        <v>0.45</v>
+      </c>
+      <c r="AK15">
+        <v>-0.62</v>
+      </c>
+      <c r="AL15">
+        <v>0.62</v>
       </c>
       <c r="AM15">
         <v>6.62</v>
@@ -2199,7 +2427,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2211,7 +2439,7 @@
         <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G16">
         <v>824560</v>
@@ -2270,17 +2498,23 @@
       <c r="Y16">
         <v>0.9809</v>
       </c>
+      <c r="Z16">
+        <v>3</v>
+      </c>
       <c r="AA16" t="s">
         <v>44</v>
       </c>
+      <c r="AB16">
+        <v>0.67</v>
+      </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD16">
         <v>5.17</v>
       </c>
       <c r="AE16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF16">
         <v>0.2072</v>
@@ -2290,6 +2524,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>-2.17</v>
+      </c>
+      <c r="AJ16">
+        <v>2.17</v>
+      </c>
+      <c r="AK16">
+        <v>-2.17</v>
+      </c>
+      <c r="AL16">
+        <v>2.17</v>
       </c>
       <c r="AM16">
         <v>5.17</v>
@@ -2300,7 +2546,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2312,13 +2558,13 @@
         <v>-160</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G17">
         <v>824073</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I17">
         <v>3</v>
@@ -2371,17 +2617,23 @@
       <c r="Y17">
         <v>0.8912</v>
       </c>
+      <c r="Z17">
+        <v>4</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>-2.04</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD17">
         <v>2.46</v>
       </c>
       <c r="AE17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF17">
         <v>0.2553</v>
@@ -2391,6 +2643,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>1.54</v>
+      </c>
+      <c r="AJ17">
+        <v>1.54</v>
+      </c>
+      <c r="AK17">
+        <v>1.54</v>
+      </c>
+      <c r="AL17">
+        <v>1.54</v>
       </c>
       <c r="AM17">
         <v>2.46</v>
@@ -2401,7 +2665,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2413,7 +2677,7 @@
         <v>-151</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G18">
         <v>824073</v>
@@ -2472,17 +2736,23 @@
       <c r="Y18">
         <v>0.9419</v>
       </c>
+      <c r="Z18">
+        <v>6</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB18">
+        <v>-0.98</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD18">
         <v>3.52</v>
       </c>
       <c r="AE18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF18">
         <v>0.1795</v>
@@ -2492,6 +2762,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>2.48</v>
+      </c>
+      <c r="AJ18">
+        <v>2.48</v>
+      </c>
+      <c r="AK18">
+        <v>2.48</v>
+      </c>
+      <c r="AL18">
+        <v>2.48</v>
       </c>
       <c r="AM18">
         <v>3.52</v>
@@ -2502,7 +2784,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2514,13 +2796,13 @@
         <v>118</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G19">
         <v>823910</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I19">
         <v>4.3</v>
@@ -2573,17 +2855,23 @@
       <c r="Y19">
         <v>0.994</v>
       </c>
+      <c r="Z19">
+        <v>5</v>
+      </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB19">
+        <v>0.24</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD19">
         <v>4.74</v>
       </c>
       <c r="AE19" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF19">
         <v>0.2618</v>
@@ -2593,6 +2881,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>0.26</v>
+      </c>
+      <c r="AJ19">
+        <v>0.26</v>
+      </c>
+      <c r="AK19">
+        <v>0.26</v>
+      </c>
+      <c r="AL19">
+        <v>0.26</v>
       </c>
       <c r="AM19">
         <v>4.74</v>
@@ -2603,7 +2903,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C20">
         <v>8.5</v>
@@ -2615,7 +2915,7 @@
         <v>-126</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G20">
         <v>823910</v>
@@ -2674,17 +2974,23 @@
       <c r="Y20">
         <v>1.1003</v>
       </c>
+      <c r="Z20">
+        <v>11</v>
+      </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB20">
+        <v>-0.67</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD20">
         <v>7.83</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.2787</v>
@@ -2694,6 +3000,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>3.17</v>
+      </c>
+      <c r="AJ20">
+        <v>3.17</v>
+      </c>
+      <c r="AK20">
+        <v>3.17</v>
+      </c>
+      <c r="AL20">
+        <v>3.17</v>
       </c>
       <c r="AM20">
         <v>7.83</v>
@@ -2704,7 +3022,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>4.5</v>
@@ -2716,7 +3034,7 @@
         <v>-133</v>
       </c>
       <c r="F21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G21">
         <v>823100</v>
@@ -2775,17 +3093,23 @@
       <c r="Y21">
         <v>0.9735</v>
       </c>
+      <c r="Z21">
+        <v>8</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB21">
+        <v>-0.36</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD21">
         <v>4.14</v>
       </c>
       <c r="AE21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF21">
         <v>0.1992</v>
@@ -2795,6 +3119,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>3.86</v>
+      </c>
+      <c r="AJ21">
+        <v>3.86</v>
+      </c>
+      <c r="AK21">
+        <v>3.86</v>
+      </c>
+      <c r="AL21">
+        <v>3.86</v>
       </c>
       <c r="AM21">
         <v>4.14</v>
@@ -2805,7 +3141,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C22">
         <v>3.5</v>
@@ -2817,13 +3153,13 @@
         <v>-105</v>
       </c>
       <c r="F22" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G22">
         <v>824718</v>
       </c>
       <c r="H22" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I22">
         <v>4</v>
@@ -2876,17 +3212,23 @@
       <c r="Y22">
         <v>0.9673</v>
       </c>
+      <c r="Z22">
+        <v>7</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB22">
+        <v>-0.82</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD22">
         <v>2.68</v>
       </c>
       <c r="AE22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF22">
         <v>0.2019</v>
@@ -2896,6 +3238,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>4.32</v>
+      </c>
+      <c r="AJ22">
+        <v>4.32</v>
+      </c>
+      <c r="AK22">
+        <v>4.32</v>
+      </c>
+      <c r="AL22">
+        <v>4.32</v>
       </c>
       <c r="AM22">
         <v>2.68</v>
@@ -2906,7 +3260,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>5.5</v>
@@ -2918,13 +3272,13 @@
         <v>-110</v>
       </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>824718</v>
       </c>
       <c r="H23" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I23">
         <v>4.4</v>
@@ -2977,17 +3331,23 @@
       <c r="Y23">
         <v>0.985</v>
       </c>
+      <c r="Z23">
+        <v>6</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB23">
+        <v>-0.8</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>4.7</v>
       </c>
       <c r="AE23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF23">
         <v>0.2223</v>
@@ -2997,6 +3357,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>1.3</v>
+      </c>
+      <c r="AJ23">
+        <v>1.3</v>
+      </c>
+      <c r="AK23">
+        <v>1.3</v>
+      </c>
+      <c r="AL23">
+        <v>1.3</v>
       </c>
       <c r="AM23">
         <v>4.7</v>
@@ -3007,7 +3379,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C24">
         <v>3.5</v>
@@ -3019,7 +3391,7 @@
         <v>-115</v>
       </c>
       <c r="F24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G24">
         <v>825044</v>
@@ -3078,17 +3450,23 @@
       <c r="Y24">
         <v>0.88</v>
       </c>
+      <c r="Z24">
+        <v>1</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>-0.83</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD24">
         <v>2.67</v>
       </c>
       <c r="AE24" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF24">
         <v>0.1807</v>
@@ -3098,6 +3476,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>-1.67</v>
+      </c>
+      <c r="AJ24">
+        <v>1.67</v>
+      </c>
+      <c r="AK24">
+        <v>-1.67</v>
+      </c>
+      <c r="AL24">
+        <v>1.67</v>
       </c>
       <c r="AM24">
         <v>2.67</v>
@@ -3108,7 +3498,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>5.5</v>
@@ -3120,7 +3510,7 @@
         <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G25">
         <v>825044</v>
@@ -3179,17 +3569,23 @@
       <c r="Y25">
         <v>1.0455</v>
       </c>
+      <c r="Z25">
+        <v>3</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>1.51</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD25">
         <v>6.84</v>
       </c>
       <c r="AE25" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="AF25">
         <v>0.2337</v>
@@ -3199,6 +3595,18 @@
       </c>
       <c r="AH25">
         <v>0.17</v>
+      </c>
+      <c r="AI25">
+        <v>-3.84</v>
+      </c>
+      <c r="AJ25">
+        <v>3.84</v>
+      </c>
+      <c r="AK25">
+        <v>-4.01</v>
+      </c>
+      <c r="AL25">
+        <v>4.01</v>
       </c>
       <c r="AM25">
         <v>7.01</v>
@@ -3209,7 +3617,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C26">
         <v>4.5</v>
@@ -3221,7 +3629,7 @@
         <v>-113</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G26">
         <v>824316</v>
@@ -3280,17 +3688,23 @@
       <c r="Y26">
         <v>0.9455</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB26">
+        <v>-0.27</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD26">
         <v>4.23</v>
       </c>
       <c r="AE26" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF26">
         <v>0.1909</v>
@@ -3300,6 +3714,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>1.77</v>
+      </c>
+      <c r="AJ26">
+        <v>1.77</v>
+      </c>
+      <c r="AK26">
+        <v>1.77</v>
+      </c>
+      <c r="AL26">
+        <v>1.77</v>
       </c>
       <c r="AM26">
         <v>4.23</v>
@@ -3310,7 +3736,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C27">
         <v>3.5</v>
@@ -3322,7 +3748,7 @@
         <v>-167</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>824316</v>
@@ -3381,17 +3807,23 @@
       <c r="Y27">
         <v>0.88</v>
       </c>
+      <c r="Z27">
+        <v>2</v>
+      </c>
       <c r="AA27" t="s">
         <v>44</v>
       </c>
+      <c r="AB27">
+        <v>-0.64</v>
+      </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD27">
         <v>2.86</v>
       </c>
       <c r="AE27" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF27">
         <v>0.1924</v>
@@ -3401,6 +3833,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>-0.86</v>
+      </c>
+      <c r="AJ27">
+        <v>0.86</v>
+      </c>
+      <c r="AK27">
+        <v>-0.86</v>
+      </c>
+      <c r="AL27">
+        <v>0.86</v>
       </c>
       <c r="AM27">
         <v>2.86</v>
@@ -3411,7 +3855,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C28">
         <v>4.5</v>
@@ -3423,7 +3867,7 @@
         <v>-128</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G28">
         <v>823261</v>
@@ -3482,17 +3926,23 @@
       <c r="Y28">
         <v>0.9907</v>
       </c>
+      <c r="Z28">
+        <v>5</v>
+      </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>56</v>
+      </c>
+      <c r="AB28">
+        <v>-0.12</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD28">
         <v>4.38</v>
       </c>
       <c r="AE28" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF28">
         <v>0.232</v>
@@ -3502,6 +3952,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>0.62</v>
+      </c>
+      <c r="AJ28">
+        <v>0.62</v>
+      </c>
+      <c r="AK28">
+        <v>0.62</v>
+      </c>
+      <c r="AL28">
+        <v>0.62</v>
       </c>
       <c r="AM28">
         <v>4.38</v>
@@ -3512,7 +3974,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C29">
         <v>4.5</v>
@@ -3524,7 +3986,7 @@
         <v>-102</v>
       </c>
       <c r="F29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G29">
         <v>823261</v>
@@ -3583,17 +4045,23 @@
       <c r="Y29">
         <v>0.9951</v>
       </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
       <c r="AA29" t="s">
         <v>44</v>
       </c>
+      <c r="AB29">
+        <v>-0.24</v>
+      </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD29">
         <v>4.26</v>
       </c>
       <c r="AE29" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AF29">
         <v>0.2124</v>
@@ -3603,6 +4071,18 @@
       </c>
       <c r="AH29">
         <v>0</v>
+      </c>
+      <c r="AI29">
+        <v>-4.26</v>
+      </c>
+      <c r="AJ29">
+        <v>4.26</v>
+      </c>
+      <c r="AK29">
+        <v>-4.26</v>
+      </c>
+      <c r="AL29">
+        <v>4.26</v>
       </c>
       <c r="AM29">
         <v>4.26</v>
@@ -3613,7 +4093,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C30">
         <v>5.5</v>
@@ -3625,31 +4105,31 @@
         <v>130</v>
       </c>
       <c r="F30" t="s">
+        <v>55</v>
+      </c>
+      <c r="G30" t="s">
         <v>52</v>
       </c>
-      <c r="G30" t="s">
-        <v>44</v>
-      </c>
       <c r="H30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L30">
         <v>1</v>
       </c>
       <c r="S30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
@@ -3657,7 +4137,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>4.5</v>
@@ -3669,31 +4149,31 @@
         <v>104</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L31">
         <v>6</v>
       </c>
       <c r="S31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
@@ -3701,7 +4181,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>3.5</v>
@@ -3713,31 +4193,31 @@
         <v>-110</v>
       </c>
       <c r="F32" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>